<commit_message>
refactor: enhance data processing with improved garbage value handling and new helper functions
</commit_message>
<xml_diff>
--- a/Dữ liệu mẫu/Mapping.xlsx
+++ b/Dữ liệu mẫu/Mapping.xlsx
@@ -2012,7 +2012,7 @@
 3. Ghi kết quả vào: data.summary.sections[order=3].latestBySpecialty[].trends[].name</t>
   </si>
   <si>
-    <t>trends[].name = tên chỉ số được so sánh | Lưu ý: chỉ Huyết áp, Cân nặng và chỉ số lab có dữ liệu ở cả hai lượt; không tự tạo tên.</t>
+    <t>trends[].name = tên chỉ số được so sánh | Lưu ý: chỉ Huyết áp, Cân nặng,  và chỉ số lab(Cận lâm sàn) có dữ liệu ở cả hai lượt; không tự tạo tên.</t>
   </si>
   <si>
     <t>data.summary.sections[order=3].latestBySpecialty[].trends[].from</t>
@@ -7163,12 +7163,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
+  <sheetPr/>
   <dimension ref="A1:N100"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.85185185185185" style="16" customWidth="1"/>
-    <col min="2" max="2" width="45.8518518518519" style="16" customWidth="1"/>
+    <col min="2" max="2" width="73.3240740740741" style="16" customWidth="1"/>
     <col min="3" max="3" width="18.712962962963" style="16" customWidth="1"/>
     <col min="4" max="4" width="50" style="16" customWidth="1"/>
     <col min="5" max="5" width="14.712962962963" style="16" customWidth="1"/>
@@ -7178,7 +7178,9 @@
     <col min="10" max="10" width="53.5740740740741" style="16" customWidth="1"/>
     <col min="11" max="11" width="41.5740740740741" style="16" customWidth="1"/>
     <col min="12" max="12" width="62" style="16" customWidth="1"/>
-    <col min="13" max="16384" width="9.13888888888889" style="16" customWidth="1"/>
+    <col min="13" max="13" width="9.13888888888889" style="16" customWidth="1"/>
+    <col min="14" max="14" width="33.4907407407407" style="16" customWidth="1"/>
+    <col min="15" max="16384" width="9.13888888888889" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -7374,7 +7376,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="6" s="14" customFormat="1" ht="409.5" hidden="1" customHeight="1" spans="1:13">
+    <row r="6" s="14" customFormat="1" ht="409.5" customHeight="1" spans="1:13">
       <c r="A6" s="23">
         <v>5</v>
       </c>
@@ -7410,7 +7412,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" s="14" customFormat="1" ht="336" hidden="1" customHeight="1" spans="1:13">
+    <row r="7" s="14" customFormat="1" ht="336" customHeight="1" spans="1:13">
       <c r="A7" s="23">
         <v>6</v>
       </c>
@@ -7484,7 +7486,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="9" s="14" customFormat="1" ht="152.25" hidden="1" customHeight="1" spans="1:13">
+    <row r="9" s="14" customFormat="1" ht="152.25" customHeight="1" spans="1:13">
       <c r="A9" s="23">
         <v>8</v>
       </c>
@@ -7521,7 +7523,7 @@
       </c>
       <c r="M9" s="34"/>
     </row>
-    <row r="10" s="14" customFormat="1" ht="244.5" hidden="1" customHeight="1" spans="1:13">
+    <row r="10" s="14" customFormat="1" ht="244.5" customHeight="1" spans="1:13">
       <c r="A10" s="23">
         <v>9</v>
       </c>
@@ -7558,7 +7560,7 @@
       </c>
       <c r="M10" s="34"/>
     </row>
-    <row r="11" s="14" customFormat="1" ht="60.75" hidden="1" customHeight="1" spans="1:13">
+    <row r="11" s="14" customFormat="1" ht="60.75" customHeight="1" spans="1:13">
       <c r="A11" s="23">
         <v>10</v>
       </c>
@@ -7595,7 +7597,7 @@
       </c>
       <c r="M11" s="34"/>
     </row>
-    <row r="12" ht="106.5" hidden="1" customHeight="1" spans="1:13">
+    <row r="12" ht="106.5" customHeight="1" spans="1:13">
       <c r="A12" s="23">
         <v>11</v>
       </c>
@@ -7632,7 +7634,7 @@
       </c>
       <c r="M12" s="35"/>
     </row>
-    <row r="13" ht="137.25" hidden="1" customHeight="1" spans="1:13">
+    <row r="13" ht="137.25" customHeight="1" spans="1:13">
       <c r="A13" s="23">
         <v>12</v>
       </c>
@@ -7742,7 +7744,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="16" ht="409.5" hidden="1" customHeight="1" spans="1:13">
+    <row r="16" ht="409.5" customHeight="1" spans="1:13">
       <c r="A16" s="23">
         <v>15</v>
       </c>
@@ -7778,7 +7780,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="17" ht="121.5" hidden="1" customHeight="1" spans="1:13">
+    <row r="17" ht="121.5" customHeight="1" spans="1:13">
       <c r="A17" s="23">
         <v>16</v>
       </c>
@@ -7817,7 +7819,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="18" ht="198" hidden="1" customHeight="1" spans="1:13">
+    <row r="18" ht="198" customHeight="1" spans="1:13">
       <c r="A18" s="23">
         <v>17</v>
       </c>
@@ -7853,7 +7855,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="19" ht="183" hidden="1" customHeight="1" spans="1:13">
+    <row r="19" ht="183" customHeight="1" spans="1:13">
       <c r="A19" s="23">
         <v>18</v>
       </c>
@@ -7889,7 +7891,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="20" ht="183" hidden="1" customHeight="1" spans="1:13">
+    <row r="20" ht="183" customHeight="1" spans="1:13">
       <c r="A20" s="23">
         <v>19</v>
       </c>
@@ -8802,7 +8804,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="44" ht="305.25" hidden="1" customHeight="1" spans="1:13">
+    <row r="44" ht="305.25" customHeight="1" spans="1:13">
       <c r="A44" s="23">
         <v>43</v>
       </c>
@@ -8838,7 +8840,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="45" ht="305.25" hidden="1" customHeight="1" spans="1:13">
+    <row r="45" ht="305.25" customHeight="1" spans="1:13">
       <c r="A45" s="23">
         <v>44</v>
       </c>
@@ -9026,7 +9028,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="50" ht="229.5" hidden="1" customHeight="1" spans="1:14">
+    <row r="50" ht="229.5" customHeight="1" spans="1:14">
       <c r="A50" s="23">
         <v>49</v>
       </c>
@@ -9062,7 +9064,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="51" ht="229.5" hidden="1" customHeight="1" spans="1:14">
+    <row r="51" ht="229.5" customHeight="1" spans="1:14">
       <c r="A51" s="23">
         <v>50</v>
       </c>
@@ -9098,7 +9100,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="52" ht="290.25" hidden="1" customHeight="1" spans="1:14">
+    <row r="52" ht="290.25" customHeight="1" spans="1:14">
       <c r="A52" s="23">
         <v>51</v>
       </c>
@@ -9576,7 +9578,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="64" ht="229.5" hidden="1" customHeight="1" spans="1:14">
+    <row r="64" ht="229.5" customHeight="1" spans="1:14">
       <c r="A64" s="23">
         <v>63</v>
       </c>
@@ -9802,7 +9804,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="70" ht="121.5" hidden="1" customHeight="1" spans="1:12">
+    <row r="70" ht="121.5" customHeight="1" spans="1:12">
       <c r="A70" s="23">
         <v>69</v>
       </c>
@@ -9952,7 +9954,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="74" ht="409.5" hidden="1" customHeight="1" spans="1:12">
+    <row r="74" ht="409.5" customHeight="1" spans="1:12">
       <c r="A74" s="23">
         <v>73</v>
       </c>
@@ -9988,7 +9990,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="75" ht="305.25" hidden="1" customHeight="1" spans="1:12">
+    <row r="75" ht="305.25" customHeight="1" spans="1:12">
       <c r="A75" s="23">
         <v>74</v>
       </c>
@@ -10024,7 +10026,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="76" ht="351" hidden="1" customHeight="1" spans="1:12">
+    <row r="76" ht="351" customHeight="1" spans="1:12">
       <c r="A76" s="23">
         <v>75</v>
       </c>
@@ -10060,7 +10062,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="77" ht="351" hidden="1" customHeight="1" spans="1:12">
+    <row r="77" ht="351" customHeight="1" spans="1:12">
       <c r="A77" s="23">
         <v>76</v>
       </c>
@@ -10292,7 +10294,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="83" ht="381.75" hidden="1" customHeight="1" spans="1:14">
+    <row r="83" ht="381.75" customHeight="1" spans="1:14">
       <c r="A83" s="23">
         <v>82</v>
       </c>
@@ -10480,7 +10482,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="88" ht="275.25" hidden="1" customHeight="1" spans="1:14">
+    <row r="88" ht="275.25" customHeight="1" spans="1:14">
       <c r="A88" s="23">
         <v>87</v>
       </c>
@@ -10516,7 +10518,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="89" ht="409.5" hidden="1" customHeight="1" spans="1:14">
+    <row r="89" ht="409.5" customHeight="1" spans="1:14">
       <c r="A89" s="23">
         <v>88</v>
       </c>
@@ -10942,12 +10944,6 @@
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N99" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="10">
-      <filters>
-        <filter val="n/a"/>
-        <filter val="N"/>
-      </filters>
-    </filterColumn>
     <extLst/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>